<commit_message>
v1.1.0: agent tool use, period comparison, PDF export, design system
- AI analyst gains typed read-only tools (get_metric, compare_programs,
  get_measures, get_issue_summary, get_trends, get_demographics) driven
  by an agentic tool loop in the Anthropic provider
- Period-over-period comparison: headline/program deltas, deterministic
  narrative, compare CLI command, and a new Streamlit page
- Program-scoped performance measures (program: field on measures)
- PDF report export via Playwright Chromium or Microsoft Edge; offline
  HTML charts (--offline-charts); example PDF included
- Validated colorblind-safe design system applied to charts, Streamlit
  theme, and reports; tokens documented and synced to Claude Design
- MCP server (grant-assistant-mcp), Dockerfile, README screenshots
  captured headlessly, PUBLISHING.md deployment guide
- 173 tests passing; ruff, mypy, and format checks clean

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/analytics_summary.xlsx
+++ b/examples/analytics_summary.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="145">
   <si>
     <t>Total enrollments</t>
   </si>
@@ -1195,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -1207,10 +1207,11 @@
     <col min="8" max="8" width="13.7109375" customWidth="1"/>
     <col min="9" max="9" width="6.7109375" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" customWidth="1"/>
-    <col min="11" max="11" width="60.7109375" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" customWidth="1"/>
+    <col min="12" max="12" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -1242,10 +1243,13 @@
         <v>38</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -1276,11 +1280,11 @@
       <c r="J2" t="b">
         <v>0</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -1312,7 +1316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -1344,7 +1348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
         <v>42</v>
       </c>
@@ -1376,7 +1380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Fix PDF pagination and restrict gender values
PDF: charts and tables were cut off because Plotly sizes its SVGs once at
the browser viewport width, which did not match the paper. Lay the page
out at the printable width (720px = Letter minus 0.5in margins) before
printing, resize charts after load, and add print rules: @page size and
margins, break-inside avoidance for tables/cards/charts/list items,
repeated table headers, headings kept with their content, and a page
break after the cover. Verified: no elements overflow the print width,
16-page PDF renders cleanly.

Data: gender values are now Female, Male, Declined, Unknown in both the
generator and the two profiles. The controlled-value audit demo now uses
an unexpected race label instead.

Adds regression tests for the print rules and for generated data staying
inside the profile vocabularies.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/analytics_summary.xlsx
+++ b/examples/analytics_summary.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="143">
   <si>
     <t>Total enrollments</t>
   </si>
@@ -280,16 +280,10 @@
     <t>Female</t>
   </si>
   <si>
-    <t>Non-Binary</t>
-  </si>
-  <si>
-    <t>Transgender</t>
-  </si>
-  <si>
     <t>Declined</t>
   </si>
   <si>
-    <t>F</t>
+    <t>Unknown</t>
   </si>
   <si>
     <t>White</t>
@@ -313,6 +307,9 @@
     <t>Native Hawaiian or Pacific Islander</t>
   </si>
   <si>
+    <t>Caucasian</t>
+  </si>
+  <si>
     <t>Non-Hispanic/Non-Latino</t>
   </si>
   <si>
@@ -323,9 +320,6 @@
   </si>
   <si>
     <t>Yes</t>
-  </si>
-  <si>
-    <t>Unknown</t>
   </si>
   <si>
     <t>Maybe</t>
@@ -1517,7 +1511,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
@@ -1527,13 +1521,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1544,7 +1538,7 @@
         <v>84</v>
       </c>
       <c r="C2">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1555,7 +1549,7 @@
         <v>85</v>
       </c>
       <c r="C3">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1566,7 +1560,7 @@
         <v>86</v>
       </c>
       <c r="C4">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1577,29 +1571,29 @@
         <v>87</v>
       </c>
       <c r="C5">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B6" t="s">
         <v>88</v>
       </c>
       <c r="C6">
-        <v>7</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
         <v>89</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1607,10 +1601,10 @@
         <v>79</v>
       </c>
       <c r="B8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C8">
-        <v>113</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1618,10 +1612,10 @@
         <v>79</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9">
-        <v>81</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1629,10 +1623,10 @@
         <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C10">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1643,7 +1637,7 @@
         <v>92</v>
       </c>
       <c r="C11">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1654,7 +1648,7 @@
         <v>93</v>
       </c>
       <c r="C12">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1665,7 +1659,7 @@
         <v>94</v>
       </c>
       <c r="C13">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1676,18 +1670,18 @@
         <v>95</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B15" t="s">
         <v>96</v>
       </c>
       <c r="C15">
-        <v>5</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1698,7 +1692,7 @@
         <v>97</v>
       </c>
       <c r="C16">
-        <v>199</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1706,10 +1700,10 @@
         <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="C17">
-        <v>45</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1717,21 +1711,21 @@
         <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C18">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>221</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1742,7 +1736,7 @@
         <v>99</v>
       </c>
       <c r="C20">
-        <v>221</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1750,10 +1744,10 @@
         <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="C21">
-        <v>28</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1761,21 +1755,21 @@
         <v>81</v>
       </c>
       <c r="B22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C22">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>151</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1786,7 +1780,7 @@
         <v>99</v>
       </c>
       <c r="C24">
-        <v>151</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1794,21 +1788,21 @@
         <v>82</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="C25">
-        <v>97</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B26" t="s">
         <v>101</v>
       </c>
       <c r="C26">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1816,10 +1810,10 @@
         <v>83</v>
       </c>
       <c r="B27" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1827,10 +1821,10 @@
         <v>83</v>
       </c>
       <c r="B28" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C28">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1838,10 +1832,10 @@
         <v>83</v>
       </c>
       <c r="B29" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C29">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1849,10 +1843,10 @@
         <v>83</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C30">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1860,10 +1854,10 @@
         <v>83</v>
       </c>
       <c r="B31" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C31">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1871,10 +1865,10 @@
         <v>83</v>
       </c>
       <c r="B32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C32">
-        <v>39</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1882,20 +1876,9 @@
         <v>83</v>
       </c>
       <c r="B33" t="s">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="C33">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" t="s">
-        <v>101</v>
-      </c>
-      <c r="C34">
         <v>2</v>
       </c>
     </row>
@@ -1915,15 +1898,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B2">
         <v>23</v>
@@ -1931,7 +1914,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B3">
         <v>23</v>
@@ -1939,7 +1922,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B4">
         <v>21</v>
@@ -1947,7 +1930,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B5">
         <v>13</v>
@@ -1955,7 +1938,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B6">
         <v>13</v>
@@ -1963,7 +1946,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -1971,7 +1954,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -1979,7 +1962,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B9">
         <v>6</v>
@@ -1987,7 +1970,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B10">
         <v>5</v>
@@ -1995,7 +1978,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B11">
         <v>5</v>
@@ -2003,7 +1986,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B12">
         <v>4</v>
@@ -2011,7 +1994,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B13">
         <v>4</v>
@@ -2019,7 +2002,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -2027,7 +2010,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -2035,7 +2018,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -2043,7 +2026,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -2066,18 +2049,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2088,7 +2071,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B3">
         <v>20</v>
@@ -2099,7 +2082,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B4">
         <v>21</v>
@@ -2110,7 +2093,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B5">
         <v>22</v>
@@ -2121,7 +2104,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B6">
         <v>18</v>
@@ -2132,7 +2115,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B7">
         <v>22</v>
@@ -2143,7 +2126,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B8">
         <v>19</v>
@@ -2154,7 +2137,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B9">
         <v>20</v>
@@ -2165,7 +2148,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B10">
         <v>22</v>
@@ -2176,7 +2159,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B11">
         <v>34</v>
@@ -2187,7 +2170,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B12">
         <v>21</v>
@@ -2198,7 +2181,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B13">
         <v>20</v>
@@ -2209,7 +2192,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B14">
         <v>20</v>

</xml_diff>

<commit_message>
v1.6.1: route chat responses automatically, rename example grants
The chat asked the user to pick streaming vs tool lookup, but they had no way
to know which a question needed. should_stream now routes by intent — narrative
questions stream, everything else (including unrecognized) takes the traced
tool loop — and the toggle became Automatic / Always stream / Always tools.

Example grants renamed to Stable Homes and Bridge to Home (display name only;
profile_id unchanged), the selector now shows the grant name, and all
committed artifacts regenerated to match.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/analytics_summary.xlsx
+++ b/examples/analytics_summary.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="146">
   <si>
     <t>Total enrollments</t>
   </si>
@@ -139,6 +139,9 @@
     <t>small_sample</t>
   </si>
   <si>
+    <t>median_length_of_stay_days</t>
+  </si>
+  <si>
     <t>HS-1</t>
   </si>
   <si>
@@ -218,6 +221,12 @@
   </si>
   <si>
     <t>description</t>
+  </si>
+  <si>
+    <t>attainment_pct</t>
+  </si>
+  <si>
+    <t>period_elapsed_pct</t>
   </si>
   <si>
     <t>3_month</t>
@@ -1000,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -1016,9 +1025,10 @@
     <col min="11" max="11" width="22.7109375" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" customWidth="1"/>
     <col min="13" max="13" width="14.7109375" customWidth="1"/>
+    <col min="14" max="14" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -1058,8 +1068,11 @@
       <c r="M1" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="N1" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -1099,8 +1112,11 @@
       <c r="M2" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:13">
+      <c r="N2">
+        <v>94.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1140,8 +1156,11 @@
       <c r="M3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:13">
+      <c r="N3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1180,6 +1199,9 @@
       </c>
       <c r="M4" t="b">
         <v>0</v>
+      </c>
+      <c r="N4">
+        <v>63.5</v>
       </c>
     </row>
   </sheetData>
@@ -1189,7 +1211,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -1203,35 +1225,37 @@
     <col min="10" max="10" width="14.7109375" customWidth="1"/>
     <col min="11" max="11" width="9.7109375" customWidth="1"/>
     <col min="12" max="12" width="60.7109375" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>38</v>
@@ -1240,24 +1264,30 @@
         <v>26</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
+        <v>66</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F2">
         <v>60</v>
@@ -1275,24 +1305,30 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2">
+        <v>106.8</v>
+      </c>
+      <c r="N2">
+        <v>211.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" t="s">
         <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" t="s">
-        <v>54</v>
       </c>
       <c r="F3">
         <v>40</v>
@@ -1309,22 +1345,28 @@
       <c r="J3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:12">
+      <c r="M3">
+        <v>117</v>
+      </c>
+      <c r="N3">
+        <v>211.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F4">
         <v>70</v>
@@ -1341,22 +1383,28 @@
       <c r="J4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="M4">
+        <v>138.9</v>
+      </c>
+      <c r="N4">
+        <v>211.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F5">
         <v>90</v>
@@ -1373,22 +1421,28 @@
       <c r="J5" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:12">
+      <c r="M5">
+        <v>109.8</v>
+      </c>
+      <c r="N5">
+        <v>211.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F6">
         <v>85</v>
@@ -1404,6 +1458,12 @@
       </c>
       <c r="J6" t="b">
         <v>0</v>
+      </c>
+      <c r="M6">
+        <v>115.2</v>
+      </c>
+      <c r="N6">
+        <v>211.5</v>
       </c>
     </row>
   </sheetData>
@@ -1426,30 +1486,30 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C2">
         <v>145</v>
@@ -1466,10 +1526,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C3">
         <v>145</v>
@@ -1486,10 +1546,10 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C4">
         <v>145</v>
@@ -1521,21 +1581,21 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C2">
         <v>122</v>
@@ -1543,10 +1603,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C3">
         <v>121</v>
@@ -1554,10 +1614,10 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C4">
         <v>10</v>
@@ -1565,10 +1625,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C5">
         <v>7</v>
@@ -1576,10 +1636,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C6">
         <v>113</v>
@@ -1587,10 +1647,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C7">
         <v>81</v>
@@ -1598,10 +1658,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C8">
         <v>18</v>
@@ -1609,10 +1669,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C9">
         <v>16</v>
@@ -1620,10 +1680,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C10">
         <v>12</v>
@@ -1631,10 +1691,10 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C11">
         <v>9</v>
@@ -1642,10 +1702,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C12">
         <v>5</v>
@@ -1653,10 +1713,10 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C13">
         <v>5</v>
@@ -1664,10 +1724,10 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1675,10 +1735,10 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B15" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C15">
         <v>199</v>
@@ -1686,10 +1746,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C16">
         <v>45</v>
@@ -1697,10 +1757,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C17">
         <v>11</v>
@@ -1708,10 +1768,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B18" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C18">
         <v>5</v>
@@ -1719,10 +1779,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C19">
         <v>221</v>
@@ -1730,10 +1790,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B20" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C20">
         <v>28</v>
@@ -1741,10 +1801,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C21">
         <v>10</v>
@@ -1752,10 +1812,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1763,10 +1823,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B23" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C23">
         <v>151</v>
@@ -1774,10 +1834,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B24" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C24">
         <v>97</v>
@@ -1785,10 +1845,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C25">
         <v>12</v>
@@ -1796,10 +1856,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -1807,10 +1867,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B27" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C27">
         <v>34</v>
@@ -1818,10 +1878,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B28" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C28">
         <v>38</v>
@@ -1829,10 +1889,10 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B29" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C29">
         <v>42</v>
@@ -1840,10 +1900,10 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B30" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C30">
         <v>45</v>
@@ -1851,10 +1911,10 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B31" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C31">
         <v>39</v>
@@ -1862,10 +1922,10 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B32" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C32">
         <v>60</v>
@@ -1873,10 +1933,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -1898,15 +1958,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B2">
         <v>23</v>
@@ -1914,7 +1974,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B3">
         <v>23</v>
@@ -1922,7 +1982,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B4">
         <v>21</v>
@@ -1930,7 +1990,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B5">
         <v>13</v>
@@ -1938,7 +1998,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B6">
         <v>13</v>
@@ -1946,7 +2006,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -1954,7 +2014,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -1962,7 +2022,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B9">
         <v>6</v>
@@ -1970,7 +2030,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B10">
         <v>5</v>
@@ -1978,7 +2038,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B11">
         <v>5</v>
@@ -1986,7 +2046,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B12">
         <v>4</v>
@@ -1994,7 +2054,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B13">
         <v>4</v>
@@ -2002,7 +2062,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -2010,7 +2070,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -2018,7 +2078,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -2026,7 +2086,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -2049,18 +2109,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2071,7 +2131,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B3">
         <v>20</v>
@@ -2082,7 +2142,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B4">
         <v>21</v>
@@ -2093,7 +2153,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B5">
         <v>22</v>
@@ -2104,7 +2164,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B6">
         <v>18</v>
@@ -2115,7 +2175,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B7">
         <v>22</v>
@@ -2126,7 +2186,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B8">
         <v>19</v>
@@ -2137,7 +2197,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B9">
         <v>20</v>
@@ -2148,7 +2208,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B10">
         <v>22</v>
@@ -2159,7 +2219,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B11">
         <v>34</v>
@@ -2170,7 +2230,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B12">
         <v>21</v>
@@ -2181,7 +2241,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B13">
         <v>20</v>
@@ -2192,7 +2252,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B14">
         <v>20</v>

</xml_diff>